<commit_message>
Cambia el dominio de correo de prueba y evita abrir el home en la compra
- GeneradorDatos: los usuarios de prueba usan el dominio @carlosmail.com.
- SeleccionarProducto: toma la categoría del menú de la página actual en
  lugar de abrir el home, cuyo evento load superó los 3 minutos en una
  ejecución y agotó el tiempo de espera de Selenium.
- README, Excel y evidencias actualizados con la ejecución del 14-10-2026
  (3/3 escenarios exitosos); nuevo hallazgo H-05 sobre la carga del home.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Plan_Pruebas_BonBonite.xlsx
+++ b/Plan_Pruebas_BonBonite.xlsx
@@ -1674,7 +1674,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Datos dinámicos generados en cada ejecución (Datafaker): cédula única de 10 dígitos que empieza por 9 y correo qa.auto.&lt;timestamp&gt;@mailinator.com para identificar las cuentas de la automatización. El producto no está quemado: se elige el primero de la categoría con talla en inventario.</t>
+          <t>Datos dinámicos generados en cada ejecución (Datafaker): cédula única de 10 dígitos que empieza por 9 y correo qa.auto.&lt;timestamp&gt;@carlosmail.com para identificar las cuentas de la automatización. El producto no está quemado: se elige el primero de la categoría con talla en inventario.</t>
         </is>
       </c>
       <c r="C31" s="6" t="n"/>
@@ -2507,7 +2507,7 @@
           <t>Generados en cada ejecución (GeneradorDatos):
 • Nombres: Laura · Apellidos: aleatorio
 • Cédula: 10 dígitos únicos que empiezan por 9
-• Correo: qa.auto.&lt;timestamp&gt;@mailinator.com
+• Correo: qa.auto.&lt;timestamp&gt;@carlosmail.com
 • Contraseña: QaAuto#&lt;timestamp&gt;
 • Autorización de tratamiento de datos: marcada</t>
         </is>
@@ -2542,7 +2542,7 @@
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>18.2</v>
+        <v>23.3</v>
       </c>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 01:02:00 (America/Bogota)</t>
+          <t>2026-10-14 02:03:34 (America/Bogota)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
@@ -2689,7 +2689,7 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>7.3</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="23" ht="27" customHeight="1">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>• Laura se registra con los datos Laura Guillen (cédula 9957720959, qa.auto.1791957720959@mailinator.com)</t>
+          <t>• Laura se registra con los datos Laura Rocha (cédula 9961414194, qa.auto.1791961414194@carlosmail.com)</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="24" ht="54" customHeight="1">
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -3184,7 +3184,7 @@
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>37.5</v>
+        <v>47.3</v>
       </c>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 01:01:23 (America/Bogota)</t>
+          <t>2026-10-14 02:02:46 (America/Bogota)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
@@ -3317,9 +3317,9 @@
       <c r="C22" s="5" t="inlineStr">
         <is>
           <t>• Sofia abre la sección Mi cuenta del sitio Bon-bonite
-• Sofia se registra con los datos Sofia Adorno (cédula 9957683177, qa.auto.1791957683177@mailinator.com)
+• Sofia se registra con los datos Sofia Roybal (cédula 9961366396, qa.auto.1791961366396@carlosmail.com)
 • Sofia cierra sesión
-• Sofia inicia sesión con la cédula y contraseña de Sofia Adorno (cédula 9957683177, qa.auto.1791957683177@mailinator.com)</t>
+• Sofia inicia sesión con la cédula y contraseña de Sofia Roybal (cédula 9961366396, qa.auto.1791961366396@carlosmail.com)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -3338,7 +3338,7 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>29.6</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="23" ht="40.5" customHeight="1">
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>5.4</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="24" ht="40.5" customHeight="1">
@@ -3404,7 +3404,7 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="25" ht="108" customHeight="1">
@@ -3440,7 +3440,7 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -3836,7 +3836,7 @@
         </is>
       </c>
       <c r="B13" s="16" t="n">
-        <v>77.7</v>
+        <v>84.8</v>
       </c>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
@@ -3852,7 +3852,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14 01:00:05 (America/Bogota)</t>
+          <t>2026-10-14 02:01:21 (America/Bogota)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n"/>
@@ -3968,9 +3968,9 @@
       <c r="C22" s="5" t="inlineStr">
         <is>
           <t>• Valentina abre la sección Mi cuenta del sitio Bon-bonite
-• Valentina se registra con los datos Valentina Nieves (cédula 9957605333, qa.auto.1791957605333@mailinator.com)
+• Valentina se registra con los datos Valentina Abrego (cédula 9961281273, qa.auto.1791961281273@carlosmail.com)
 • Valentina cierra sesión
-• Valentina inicia sesión con la cédula y contraseña de Valentina Nieves (cédula 9957605333, qa.auto.1791957605333@mailinator.com)</t>
+• Valentina inicia sesión con la cédula y contraseña de Valentina Abrego (cédula 9961281273, qa.auto.1791961281273@carlosmail.com)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -3989,7 +3989,7 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>32.1</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="23" ht="27" customHeight="1">
@@ -4022,7 +4022,7 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>24.1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" ht="27" customHeight="1">
@@ -4055,7 +4055,7 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>14.1</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="25" ht="108" customHeight="1">
@@ -4091,7 +4091,7 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="26" ht="54" customHeight="1">
@@ -4124,7 +4124,7 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>6.6</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="27" ht="121.5" customHeight="1">
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
@@ -4382,7 +4382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4564,6 +4564,38 @@
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Habilitar un ambiente de staging con pasarela en modo sandbox para cubrir el pago de punta a punta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="67.5" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>H-05</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>La página de inicio tarda más de un minuto en terminar de cargar (evento load); en una ejecución superó los 3 minutos y el navegador agotó su tiempo de espera. El HTML llega en menos de 1 s, así que la demora está en los recursos que se cargan después (la página incluye contenido multimedia y un feed de Instagram).</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Rendimiento</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Medir la página con Lighthouse o PageSpeed para identificar los recursos lentos y aplicarles carga diferida (lazy loading).</t>
         </is>
       </c>
     </row>

</xml_diff>